<commit_message>
COCINA MLV: cambios de GuiGui del 28/10, 15 etiquetas a reimprimir
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UqhgptvH9sQRGmqWbSErRY
</commit_message>
<xml_diff>
--- a/PENDRIVE/12_COCINA_MLV/lista_corte.xlsx
+++ b/PENDRIVE/12_COCINA_MLV/lista_corte.xlsx
@@ -2669,25 +2669,25 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>COCINA MLV_Alacena doble_Fondo 964x840.5x5</t>
+          <t>COCINA MLV_Alacena doble_Fondo 974x850.5x5</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>COCINA MLV_Alacena doble_Fondo 964x840.5x5</t>
+          <t>COCINA MLV_Alacena doble_Fondo 974x850.5x5</t>
         </is>
       </c>
       <c r="D25" t="n">
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>840.5</v>
+        <v>850.5</v>
       </c>
       <c r="F25" t="n">
-        <v>964</v>
+        <v>974</v>
       </c>
       <c r="G25" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.83</v>
       </c>
       <c r="H25" t="n">
         <v>5</v>
@@ -2698,13 +2698,13 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>840.5</v>
+        <v>850.5</v>
       </c>
       <c r="K25" t="n">
-        <v>964</v>
+        <v>974</v>
       </c>
       <c r="L25" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.83</v>
       </c>
       <c r="M25" t="n">
         <v>5</v>
@@ -2745,7 +2745,7 @@
       <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr">
         <is>
-          <t>Alacena doble_Fondo 964x840.5x5</t>
+          <t>Alacena doble_Fondo 974x850.5x5</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
@@ -6520,7 +6520,7 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="K67" t="n">
         <v>964</v>
@@ -6538,7 +6538,7 @@
       </c>
       <c r="O67" t="inlineStr"/>
       <c r="P67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q67" t="n">
         <v>1</v>
@@ -6673,25 +6673,25 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>COCINA MLV_Bajo mesada doble c/cesto_Fondo 974x232x5</t>
+          <t>COCINA MLV_Bajo mesada doble c/cesto_Fondo 974x227x5</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>COCINA MLV_Bajo mesada doble c/cesto_Fondo 974x232x5</t>
+          <t>COCINA MLV_Bajo mesada doble c/cesto_Fondo 974x227x5</t>
         </is>
       </c>
       <c r="D69" t="n">
         <v>1</v>
       </c>
       <c r="E69" t="n">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="F69" t="n">
         <v>974</v>
       </c>
       <c r="G69" t="n">
-        <v>0.23</v>
+        <v>0.22</v>
       </c>
       <c r="H69" t="n">
         <v>5</v>
@@ -6702,13 +6702,13 @@
         </is>
       </c>
       <c r="J69" t="n">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="K69" t="n">
         <v>974</v>
       </c>
       <c r="L69" t="n">
-        <v>0.23</v>
+        <v>0.22</v>
       </c>
       <c r="M69" t="n">
         <v>5</v>
@@ -6749,7 +6749,7 @@
       <c r="W69" t="inlineStr"/>
       <c r="X69" t="inlineStr">
         <is>
-          <t>Bajo mesada doble c/cesto_Fondo 974x232x5</t>
+          <t>Bajo mesada doble c/cesto_Fondo 974x227x5</t>
         </is>
       </c>
       <c r="Y69" t="inlineStr">
@@ -10247,7 +10247,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>18_NPetfrente_Gris</t>
+          <t>18_NEstructura_Gris</t>
         </is>
       </c>
       <c r="J108" t="n">
@@ -10338,7 +10338,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>18_NPetfrente_Gris</t>
+          <t>18_NEstructura_Gris</t>
         </is>
       </c>
       <c r="J109" t="n">
@@ -10429,7 +10429,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>18_NPetfrente_Gris</t>
+          <t>18_NEstructura_Gris</t>
         </is>
       </c>
       <c r="J110" t="n">
@@ -10520,7 +10520,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>18_NPetfrente_Gris</t>
+          <t>18_NEstructura_Gris</t>
         </is>
       </c>
       <c r="J111" t="n">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>18_NPetfrente_Gris</t>
+          <t>18_NEstructura_Gris</t>
         </is>
       </c>
       <c r="J112" t="n">
@@ -10702,7 +10702,7 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>18_NPetfrente_Gris</t>
+          <t>18_NEstructura_Gris</t>
         </is>
       </c>
       <c r="J113" t="n">

</xml_diff>